<commit_message>
Datos: Excel semilla de RELEVO_GEN y PATATA con euskera completo
Actualiza los Excel semilla de datos/ con los campos en euskera rellenos
al 100% en actuaciones e indicadores (antes solo los ambitos tenian eu).
Asi una carga en limpio de la BD local ya trae el bilinguismo completo y
permite verificar en local el cambio de idioma es/eu en todas las paginas.

No cambia codigo ni esquema; solo datos semilla.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/Plan_Sectorial_Patata.xlsx
+++ b/datos/Plan_Sectorial_Patata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\seguimiento_planes\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u0899rpe\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{016D3423-9977-45C5-A2A7-C63E2E06A341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{629A63A9-D239-4DD5-A327-9D2F9B209B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="38596" windowHeight="21075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11235" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -285,7 +285,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="305">
   <si>
     <t>Plan Sectorial — Patata de Consumo y Siembra en Euskadi</t>
   </si>
@@ -1002,6 +1002,239 @@
   </si>
   <si>
     <t>(El plan está recién publicado. Las anotaciones de seguimiento se irán generando en la aplicación a medida que avancen las actuaciones.)</t>
+  </si>
+  <si>
+    <t>HAZIren Behatokiaren bidez ad hoc ezagutza sortzea</t>
+  </si>
+  <si>
+    <t>Sektorerako prestakuntza-programak</t>
+  </si>
+  <si>
+    <t>I+G+Bren garapena landa-eremuan</t>
+  </si>
+  <si>
+    <t>Barne-ezagutza trukatzea</t>
+  </si>
+  <si>
+    <t>Ikuskatzaile talde espezializatuaren laguntza</t>
+  </si>
+  <si>
+    <t>Proiektu pilotuak/erakusleak</t>
+  </si>
+  <si>
+    <t>I+G+b arloko akordio estrategikoak</t>
+  </si>
+  <si>
+    <t>Minituberkuluen aseguramendua</t>
+  </si>
+  <si>
+    <t>Nekazaritza eta ingurumeneko laguntzak mantentzea</t>
+  </si>
+  <si>
+    <t>Produktu fitosanitarioak etengabeko berrikustea</t>
+  </si>
+  <si>
+    <t>Uraren erabilera optimizazioa</t>
+  </si>
+  <si>
+    <t>Patataren nekazaritza-aseguruaren kontratazioa sustatzea</t>
+  </si>
+  <si>
+    <t>Patataren sektorean gazteak sartzea</t>
+  </si>
+  <si>
+    <t>Eskulaneko baliabideen zuzkidura</t>
+  </si>
+  <si>
+    <t>Modernizazioan inbertitzea</t>
+  </si>
+  <si>
+    <t>Inbertsio berritzailea/teknologikoa</t>
+  </si>
+  <si>
+    <t>Makinen erabilera partekatua sustatzea</t>
+  </si>
+  <si>
+    <t>Laguntzen irisgarritasun unibertsala</t>
+  </si>
+  <si>
+    <t>Produktua kudeatzeko, kontserbatzeko eta balioztatzeko inbertsioak</t>
+  </si>
+  <si>
+    <t>"Patata de Álava – Arabako Patata" BJD bultzatzea</t>
+  </si>
+  <si>
+    <t>Kontsumorako patataren sustapena</t>
+  </si>
+  <si>
+    <t>Merkatu-eskari berriak</t>
+  </si>
+  <si>
+    <t>Sinplifikazio administratiboa</t>
+  </si>
+  <si>
+    <t>Sektorearen egituraketa</t>
+  </si>
+  <si>
+    <t>Patataren sektoreko elkarrizketa-foroa</t>
+  </si>
+  <si>
+    <t>Idazkaritza Teknikoa</t>
+  </si>
+  <si>
+    <t>Aginte-mahai</t>
+  </si>
+  <si>
+    <t>Aginte-taula operatibo batean egituratutako funtsezko adierazleen multzo bat definitzea, ekintzen betetze-maila eta sektorearen gaineko benetako eragina ebaluatu ahal izateko.</t>
+  </si>
+  <si>
+    <t>Eusko Jaurlaritzaren ardurapeko unitate operatiboa, aurreikusitako ekintzak koordinatzen dituena eta Gobernantzaren esparrua dinamizatzen duena, jarraitutasuna, gardentasuna eta koordinazioa ziurtatuz.</t>
+  </si>
+  <si>
+    <t>Dagoen lan-foroaren (Patataren Mahaia) jarduera eta dinamismo handiagoa, sektore ekoizlearen eta administrazioaren arteko elkarrizketa-foro gisa, sektorearen hobekuntza-planak diagnostikatzeko, adosteko, garatzeko eta abian jartzeko.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sektorearen antolaketa indartzea elkarte- edo enpresa-formulen bidez: baliabide materialak (hala nola traktoreak eta makineria) kontzentratzeko, elkarri laguntzeko eta bateratzeko prozesuak.
+</t>
+  </si>
+  <si>
+    <t>Ekoizleei zuzendutako ekintza pedagogikoa eta dibulgaziokoa, nekazaritza-aseguruaren ulermena eta kontratazioa hobetzeko.</t>
+  </si>
+  <si>
+    <t>Lurraldean baliabide hidrikoen erabilera orekatua ziurtatzea eta egungo eskubiderik gabeko ustiategiak ureztatzeko aukera erraztea, ureztatzaileen komunitateen bidez. Gutxiegi erabilitako azpiegitura hidraulikoak saihestea.</t>
+  </si>
+  <si>
+    <t>Gomendatutako fitosanitarioen katalogo tekniko bat urtero eguneratzea, bereziki birosien aurrean, izurriteen erabilera integratua eta tratamenduko emaitzen hobekuntza erraztuz.</t>
+  </si>
+  <si>
+    <t>Hazitarako patataren laborea NPBren nekazaritza-ingurumeneko eskemetan sartzea, nekazaritzako txandakatze iraunkorrak eta osasun-baldintza onak saritzeko.</t>
+  </si>
+  <si>
+    <t>Inbertsioa azpiegituretan (negutegi automatizatuak, aklimatazio-ganberak) minituberkulu osasuntsuak, genetikoki kontrolatuak eta aklimatatuak ekoizteko. Neikerren egungo azpiegituren dimentsionamendua.</t>
+  </si>
+  <si>
+    <t>Aliantzak erreferentziazko nazioarteko erakundeekin (Neiker bidez), material genetikoa, barietate komertzial berriak eta metodologia aurreratuak eskuratzeko. European Association for Potato Research (EAPR) foroetan parte hartzea.</t>
+  </si>
+  <si>
+    <t>Lurralde- eta partaidetza-ikuspegia duten plan pilotuak, tokiko nekazariekin, teknika berriak baliozkotzeko, izurriteak, barietateak eta merkataritza-eskemak hautemateko. Iturrietako etxalde esperimentalean itsasargi finka bat garatzea, erakustoki iraunkor gisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazitarako patatarentzako berariazko ikuskapen-talde bat ziurtatzea, teknikoki hornitua eta eguneratua, eginkizun bikoitzarekin: kalitate-kontrola/landare-osasuna eta ekoizleei etengabeko laguntza teknikoa ematea.
+</t>
+  </si>
+  <si>
+    <t>Hazitarako patataren azalera</t>
+  </si>
+  <si>
+    <t>Kontsumorako patataren azalera</t>
+  </si>
+  <si>
+    <t>Hazitarako patataren errendimendua</t>
+  </si>
+  <si>
+    <t>Kontsumorako patataren errendimendua</t>
+  </si>
+  <si>
+    <t>Gaixotasunagatik baztertutako hektareen ehunekoa</t>
+  </si>
+  <si>
+    <t>Hazitarako patataren kilogramo ziurtatuak</t>
+  </si>
+  <si>
+    <t>Arabako Patataren BJD sortzea</t>
+  </si>
+  <si>
+    <t>Arabako patata-produktuen erreferentzia kopurua merkatuan</t>
+  </si>
+  <si>
+    <t>Merkatuan dauden Arabako patatetan oinarritutako produktu bereizien kopurua (formatuak, gamak, barietate komertzialak). Mikro 3 helburuari lotua. Tarteko helmuga 2028:8 erreferentzia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rabako patatarentzat Babestutako Jatorri Deitura bat dago. 0 = sortu gabea, 1 = sortua. Mikro 3 helburuari lotuta (ekoizpen-katea merkatuaren eskarietara egokitzea).
+</t>
+  </si>
+  <si>
+    <t>Euskadin ekoitzitako hazitarako patata ziurtatuaren urteko bolumena. Mikro 2 helburuari lotua. Tarteko helmuga 2028: 7.272.375 kg. Erreferentzia: azken 5 urteetako batez bestekoa 7.166.858 kg.</t>
+  </si>
+  <si>
+    <t>Ziurtapen-prozesuan gaixotasunengatik baztertutako hazitarako patataren azaleraren ehunekoa. Mikro 2 helburuari lotua. Tarteko helmuga 2028: % 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontsumorako patataren laborantzaren batez besteko produktibitatea. Mikro 2 helburuari lotuta (kalitatea eta errendimendua handitzea).
+</t>
+  </si>
+  <si>
+    <t>Hazitarako patataren labore ziurtatuaren batez besteko produktibitatea. Mikro 2 helburuari lotuta (kalitatea eta errendimendua handitzea). Tarteko helmuga 2028: 15.375 kg/ha. Erreferentzia: azken 5 urteetako batez bestekoa 15.106 kg/ha.</t>
+  </si>
+  <si>
+    <t>Kontsumorako patata landatzeko hektareak. Mikro 1 helburuari lotuta (landatutako azalera handitzea). Tarteko helmuga 2028:800 ha.</t>
+  </si>
+  <si>
+    <t>Hazitarako patata landatzeko hektareak. Mikro 1 helburuari lotuta (landatutako azalera handitzea). Tarteko helmuga 2028:550 ha.</t>
+  </si>
+  <si>
+    <t>Arabako patataren balio-katea indartzeko plan estrategikoa, ereiteko nahiz kontsumitzeko, esku hartzeko 5 ardatzetan (ezagutza, iraunkortasuna, azpiegiturak eta ekipamendua, posizionamendua eta gobernantza) bildutako 27 jarduketaren bidez. Funtsezko helburuak: landutako azalera handitzea, kalitatea eta errendimendua hobetzea, eta ekoizpen-katea merkatuaren eskarietara egokitzea.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAZIren Behatokia sektorearen behatoki tekniko gisa zabaltzea, balio-kate osoa, diagnostiko zehatzak, joeren txostenak eta kanpainen egoera irudikatuko duen aginte-taula sinoptiko bat txertatuz, landa-datuak eta merkataritza-erreferentziak integratuz.
+[Tresna/programa: BEHATOKI HAZI] 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nekazariei eta teknikariei zuzendutako prestakuntza-programa integrala, gazteei arreta berezia eskainiz: jardunaldiak, ikastaroak eta tailerrak barietate-kudeaketari, laborantzaren erabilerari eta iraunkortasunari buruz. Mugarria: nazioarteko bokazioa duen ekoizle espezializatuaren urteko ikastaroa, EBko estandarrekin lerrokatua.
+[Arduradunkidea (k): NEIKER | Tresna/programa: FPE] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neikerren hazitarako patataren ildoa indartzea eta I+G+B plana sektore ekoizlearekin, erronka teknikoak, ingurumenekoak eta barietatekoak konpontzeko. Zehaztasun-nekazaritza barne hartzen du (sentsoreak, insumoen monitorizazioa eta optimizazioa).
+[Tresna/programa: FARO FINKA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nekazarien, teknikarien eta adituen arteko aurrez aurreko truke-espazioak eta gune digitalak. AKIS, Neikerren Berritzen Plana eta HAZIren Behatokia bezalako ekimenak babestea. Inplikazio publiko eta pribatu handiena duten bilera sektorial ohikoenak.
+[Tresna/programa: AKIS FOROA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EAEko nekazaritza-sektorean belaunaldien arteko erreleborako estrategia integralaren barruan txertaketak artikulatzea, Arabako nekazaritza-dibertsifikazioaren ardatz espezifiko gisa.
+[Arduradunkidea (k): AFA | Tresna/programa: TXANDA + DIBERTSIFIKAZIOA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sasoikako Lanaren Planari dagokionez, ereiteko eta kontsumitzeko eskulanaren beharrei heltzeko zeharkako ekintza.
+[Arduradunkidea (k): AFA | Tresna/programa: SASOIKAKO LANAREN PROGRAMA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produktibitatea hobetu eta kostuak murriztuko dituzten ustiategiak modernizatzeko foru laguntzen lerroa, segurtasuna eta ergonomia indartuz. Ureztatze eraginkorreko ekipoak, makineria espezifikoa (ereiteko makinak, paketatzeko makinak, atoiak) eta azpiegitura osagarriak barne hartzen ditu.
+[Tresna/programa: MODERNIZAZIOA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teknologia disruptiboak eta soluzio aurreratuak hartzea laborantzaren ekoizpenean eta kudeaketan (Handitu Innova edo proiektu pilotuak prozesu digital eta agronomikoetan), ingurumen-insumoak eta -inpaktua murriztera bideratuta.
+[Tresna/programa: HANDITU INNOVA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nekazaritzako makineria batera erosteko edo kudeatzeko pizgarriak (CUMAS), unitateko kostuak murriztuz, balio handiko ekipamenduak eskuratzeko erraztasunak emanez eta hurbileko ustiategien edo kooperatiben arteko lankidetza indartuz.
+[Arduradunkidea (k): SEKTOREA | Tresna/programa: CUMAS] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baldintzak eta eskakizunak egokitzea laguntzak operadore-tipologia guztietara irits daitezen: ATP, ustiategi txikiak, ekoizle berriak, kooperatibak, zerbitzu-enpresak eta ekimen kolektibizatuak.
+[Arduradunkidea (k): AFA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laguntza publikoa (Lehiatu edo beste batzuk), uzta bildu ondorengo logistika- eta kontserbazio-zentroak sortzeko eta hobetzeko. Manipulatzeko, kalibratzeko, kontserbatzeko, ontziratzeko eta trazabilitate- eta ziurtapen-sistemetan egindako inbertsioak.
+[Tresna/programa: LEHIATU INB] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arabako hazitarako patataren prestigioa eta aintzatespena berrezartzeko ekintza estrategikoa, Estatuan eta Europan kalitatezko erreferentzia gisa, irizpide teknikoak, kultura-balioak eta merkataritza-posizionamendua konbinatuz.
+[Arduradunkidea (k): HAZI] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posizionamendu-ekintza globala helburuko publikoaren arabera: elikadura-hezkuntzako programak (urtarokotasuna, barietateak, kontsumo-moduak, kalitate-bereizgarriak) eta gastronomiako eta elikagaien industriako profesionalentzako programa espezifikoak.
+[Arduradunkidea (k): EJ] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kategoria berriekin lerrokatutako eskaintza bat garatzea (IV. eta V. Gamak, izoztua, prozesatua) hurbiltasunaren, iraunkortasunaren eta 0 kilometroaren ikuspegitik. Joeren jarraipen aktiboa HAZIren Behatokiaren bidez.
+[Arduradunkidea (k): SEKTOREA] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sektoreko eragileen eta administrazio publikoen arteko harremana optimizatzea: karga burokratikoak murriztea, erakunde-rolak argitzea eta sailen eta administrazio-mailen arteko harreman-puntuak hobetzea.
+[Arduradunkidea (k): AFA] </t>
   </si>
 </sst>
 </file>
@@ -1148,8 +1381,11 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1165,9 +1401,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1471,14 +1704,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:G32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="2:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="9"/>
@@ -1487,8 +1720,8 @@
       <c r="F2" s="9"/>
       <c r="G2" s="9"/>
     </row>
-    <row r="4" spans="2:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="14" t="s">
+    <row r="4" spans="2:7" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="9"/>
@@ -1497,8 +1730,8 @@
       <c r="F4" s="9"/>
       <c r="G4" s="9"/>
     </row>
-    <row r="6" spans="2:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="B6" s="15" t="s">
+    <row r="6" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B6" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="9"/>
@@ -1507,8 +1740,8 @@
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B7" s="18" t="s">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="19" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="9"/>
@@ -1517,8 +1750,8 @@
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
     </row>
-    <row r="8" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="13" t="s">
+    <row r="8" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="14" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="9"/>
@@ -1527,8 +1760,8 @@
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
     </row>
-    <row r="9" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="13" t="s">
+    <row r="9" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="9"/>
@@ -1537,8 +1770,8 @@
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
     </row>
-    <row r="10" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="13" t="s">
+    <row r="10" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="14" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="9"/>
@@ -1547,8 +1780,8 @@
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
     </row>
-    <row r="11" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="13" t="s">
+    <row r="11" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="9"/>
@@ -1557,8 +1790,8 @@
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
     </row>
-    <row r="12" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="13" t="s">
+    <row r="12" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="14" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="9"/>
@@ -1567,8 +1800,8 @@
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
     </row>
-    <row r="13" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="13" t="s">
+    <row r="13" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="9"/>
@@ -1577,8 +1810,8 @@
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
     </row>
-    <row r="14" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="13" t="s">
+    <row r="14" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="14" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="9"/>
@@ -1587,8 +1820,8 @@
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
     </row>
-    <row r="15" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="13" t="s">
+    <row r="15" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="14" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="9"/>
@@ -1597,8 +1830,8 @@
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
     </row>
-    <row r="16" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="13" t="s">
+    <row r="16" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C16" s="9"/>
@@ -1607,8 +1840,8 @@
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
     </row>
-    <row r="17" spans="2:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="13" t="s">
+    <row r="17" spans="2:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="14" t="s">
         <v>13</v>
       </c>
       <c r="C17" s="9"/>
@@ -1617,8 +1850,8 @@
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
     </row>
-    <row r="19" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="14" t="s">
+    <row r="19" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="15" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="9"/>
@@ -1627,8 +1860,8 @@
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
     </row>
-    <row r="21" spans="2:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="B21" s="15" t="s">
+    <row r="21" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B21" s="16" t="s">
         <v>15</v>
       </c>
       <c r="C21" s="9"/>
@@ -1637,104 +1870,104 @@
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
     </row>
-    <row r="23" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="12"/>
-    </row>
-    <row r="24" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="13"/>
+    </row>
+    <row r="24" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="12"/>
-    </row>
-    <row r="25" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="12"/>
-    </row>
-    <row r="26" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="12"/>
-    </row>
-    <row r="27" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="12"/>
-    </row>
-    <row r="28" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="13"/>
+    </row>
+    <row r="28" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="12"/>
-    </row>
-    <row r="29" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="13"/>
+    </row>
+    <row r="29" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="12"/>
-    </row>
-    <row r="30" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="13"/>
+    </row>
+    <row r="30" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="12"/>
-    </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B32" s="16" t="s">
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="13"/>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="17" t="s">
         <v>32</v>
       </c>
       <c r="C32" s="9"/>
@@ -1778,7 +2011,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="3" width="38" customWidth="1"/>
@@ -1788,8 +2021,8 @@
     <col min="8" max="8" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:8" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>33</v>
       </c>
       <c r="B1" s="9"/>
@@ -1800,7 +2033,7 @@
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
     </row>
-    <row r="3" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -1826,7 +2059,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>42</v>
       </c>
@@ -1848,7 +2081,9 @@
       <c r="G4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="H4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>289</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1861,22 +2096,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="3" width="40" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>46</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
     </row>
-    <row r="3" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>47</v>
       </c>
@@ -1890,7 +2125,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>49</v>
       </c>
@@ -1904,7 +2139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>52</v>
       </c>
@@ -1918,7 +2153,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>55</v>
       </c>
@@ -1932,7 +2167,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -1946,7 +2181,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>61</v>
       </c>
@@ -1971,7 +2206,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -1979,15 +2214,15 @@
     <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
     </row>
-    <row r="3" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -2001,7 +2236,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>67</v>
       </c>
@@ -2013,7 +2248,7 @@
       </c>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>70</v>
       </c>
@@ -2025,7 +2260,7 @@
       </c>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>72</v>
       </c>
@@ -2037,7 +2272,7 @@
       </c>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>74</v>
       </c>
@@ -2049,7 +2284,7 @@
       </c>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>77</v>
       </c>
@@ -2072,22 +2307,22 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="55" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="6" max="6" width="42.28515625" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>80</v>
       </c>
       <c r="B1" s="9"/>
@@ -2101,7 +2336,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="3" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -2136,7 +2371,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="104" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="104.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>88</v>
       </c>
@@ -2146,11 +2381,15 @@
       <c r="C4" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="E4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>290</v>
+      </c>
       <c r="G4" s="5">
         <v>50000</v>
       </c>
@@ -2167,7 +2406,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="115.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="115.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>94</v>
       </c>
@@ -2177,11 +2416,15 @@
       <c r="C5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>235</v>
+      </c>
       <c r="E5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>291</v>
+      </c>
       <c r="G5" s="5">
         <v>200000</v>
       </c>
@@ -2198,7 +2441,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="92" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="92.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>97</v>
       </c>
@@ -2208,11 +2451,15 @@
       <c r="C6" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>236</v>
+      </c>
       <c r="E6" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>292</v>
+      </c>
       <c r="G6" s="5">
         <v>400000</v>
       </c>
@@ -2229,7 +2476,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="97.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="97.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>100</v>
       </c>
@@ -2239,11 +2486,15 @@
       <c r="C7" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="3"/>
+      <c r="D7" s="3" t="s">
+        <v>237</v>
+      </c>
       <c r="E7" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="F7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>293</v>
+      </c>
       <c r="G7" s="5">
         <v>6000</v>
       </c>
@@ -2260,7 +2511,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="76.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="76.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>103</v>
       </c>
@@ -2270,11 +2521,15 @@
       <c r="C8" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>238</v>
+      </c>
       <c r="E8" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>272</v>
+      </c>
       <c r="G8" s="6">
         <v>0</v>
       </c>
@@ -2291,7 +2546,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>106</v>
       </c>
@@ -2301,11 +2556,15 @@
       <c r="C9" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E9" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>271</v>
+      </c>
       <c r="G9" s="6">
         <v>0</v>
       </c>
@@ -2322,7 +2581,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="83" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="83.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>109</v>
       </c>
@@ -2332,11 +2591,15 @@
       <c r="C10" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>240</v>
+      </c>
       <c r="E10" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>270</v>
+      </c>
       <c r="G10" s="5">
         <v>400000</v>
       </c>
@@ -2353,7 +2616,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="81" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>112</v>
       </c>
@@ -2363,11 +2626,15 @@
       <c r="C11" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E11" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="F11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>269</v>
+      </c>
       <c r="G11" s="5">
         <v>1000000</v>
       </c>
@@ -2384,7 +2651,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="65" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>115</v>
       </c>
@@ -2394,11 +2661,15 @@
       <c r="C12" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>242</v>
+      </c>
       <c r="E12" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="F12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>268</v>
+      </c>
       <c r="G12" s="5">
         <v>500000</v>
       </c>
@@ -2415,7 +2686,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>118</v>
       </c>
@@ -2425,11 +2696,15 @@
       <c r="C13" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>243</v>
+      </c>
       <c r="E13" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>267</v>
+      </c>
       <c r="G13" s="6">
         <v>0</v>
       </c>
@@ -2446,7 +2721,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="82.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="82.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>121</v>
       </c>
@@ -2456,11 +2731,15 @@
       <c r="C14" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>244</v>
+      </c>
       <c r="E14" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="F14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>266</v>
+      </c>
       <c r="G14" s="6">
         <v>0</v>
       </c>
@@ -2477,7 +2756,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="55.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>124</v>
       </c>
@@ -2487,11 +2766,15 @@
       <c r="C15" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="E15" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>265</v>
+      </c>
       <c r="G15" s="6">
         <v>0</v>
       </c>
@@ -2508,7 +2791,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>127</v>
       </c>
@@ -2518,11 +2801,15 @@
       <c r="C16" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>246</v>
+      </c>
       <c r="E16" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>294</v>
+      </c>
       <c r="G16" s="5">
         <v>1000000</v>
       </c>
@@ -2539,7 +2826,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="77" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" ht="77.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>130</v>
       </c>
@@ -2549,11 +2836,15 @@
       <c r="C17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>247</v>
+      </c>
       <c r="E17" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="3"/>
+      <c r="F17" s="3" t="s">
+        <v>295</v>
+      </c>
       <c r="G17" s="6">
         <v>0</v>
       </c>
@@ -2570,7 +2861,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="100.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>133</v>
       </c>
@@ -2580,11 +2871,15 @@
       <c r="C18" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>248</v>
+      </c>
       <c r="E18" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="F18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>296</v>
+      </c>
       <c r="G18" s="6">
         <v>0</v>
       </c>
@@ -2601,7 +2896,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="88.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" ht="88.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>136</v>
       </c>
@@ -2611,11 +2906,15 @@
       <c r="C19" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>249</v>
+      </c>
       <c r="E19" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="F19" s="3"/>
+      <c r="F19" s="3" t="s">
+        <v>297</v>
+      </c>
       <c r="G19" s="5">
         <v>1500000</v>
       </c>
@@ -2632,7 +2931,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="96" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>139</v>
       </c>
@@ -2642,11 +2941,15 @@
       <c r="C20" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>250</v>
+      </c>
       <c r="E20" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="F20" s="3"/>
+      <c r="F20" s="3" t="s">
+        <v>298</v>
+      </c>
       <c r="G20" s="6">
         <v>0</v>
       </c>
@@ -2663,7 +2966,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="86" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" ht="86.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>142</v>
       </c>
@@ -2673,11 +2976,15 @@
       <c r="C21" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>251</v>
+      </c>
       <c r="E21" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="F21" s="3"/>
+      <c r="F21" s="3" t="s">
+        <v>299</v>
+      </c>
       <c r="G21" s="6">
         <v>0</v>
       </c>
@@ -2694,7 +3001,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="87" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>145</v>
       </c>
@@ -2704,11 +3011,15 @@
       <c r="C22" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="E22" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F22" s="3"/>
+      <c r="F22" s="3" t="s">
+        <v>300</v>
+      </c>
       <c r="G22" s="5">
         <v>4000000</v>
       </c>
@@ -2725,7 +3036,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="89" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" ht="89.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>148</v>
       </c>
@@ -2735,11 +3046,15 @@
       <c r="C23" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="E23" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3" t="s">
+        <v>301</v>
+      </c>
       <c r="G23" s="5">
         <v>50000</v>
       </c>
@@ -2756,7 +3071,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" ht="95.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>151</v>
       </c>
@@ -2766,11 +3081,15 @@
       <c r="C24" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="E24" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="F24" s="3"/>
+      <c r="F24" s="3" t="s">
+        <v>302</v>
+      </c>
       <c r="G24" s="5">
         <v>250000</v>
       </c>
@@ -2787,7 +3106,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="85.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:11" ht="85.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>154</v>
       </c>
@@ -2797,11 +3116,15 @@
       <c r="C25" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D25" s="3"/>
+      <c r="D25" s="3" t="s">
+        <v>255</v>
+      </c>
       <c r="E25" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F25" s="3"/>
+      <c r="F25" s="3" t="s">
+        <v>303</v>
+      </c>
       <c r="G25" s="6">
         <v>0</v>
       </c>
@@ -2818,7 +3141,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>157</v>
       </c>
@@ -2828,11 +3151,15 @@
       <c r="C26" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D26" s="3" t="s">
+        <v>256</v>
+      </c>
       <c r="E26" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="F26" s="3"/>
+      <c r="F26" s="3" t="s">
+        <v>304</v>
+      </c>
       <c r="G26" s="6">
         <v>0</v>
       </c>
@@ -2849,7 +3176,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="76.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:11" ht="76.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>160</v>
       </c>
@@ -2859,11 +3186,15 @@
       <c r="C27" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D27" s="3"/>
+      <c r="D27" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="E27" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="3"/>
+      <c r="F27" s="3" t="s">
+        <v>264</v>
+      </c>
       <c r="G27" s="6">
         <v>0</v>
       </c>
@@ -2880,7 +3211,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="82.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:11" ht="82.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>163</v>
       </c>
@@ -2890,11 +3221,15 @@
       <c r="C28" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="D28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>258</v>
+      </c>
       <c r="E28" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="F28" s="3"/>
+      <c r="F28" s="3" t="s">
+        <v>263</v>
+      </c>
       <c r="G28" s="6">
         <v>0</v>
       </c>
@@ -2911,7 +3246,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="71" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:11" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>166</v>
       </c>
@@ -2921,11 +3256,15 @@
       <c r="C29" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="3" t="s">
+        <v>259</v>
+      </c>
       <c r="E29" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F29" s="3"/>
+      <c r="F29" s="3" t="s">
+        <v>262</v>
+      </c>
       <c r="G29" s="6">
         <v>0</v>
       </c>
@@ -2942,7 +3281,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>169</v>
       </c>
@@ -2952,11 +3291,15 @@
       <c r="C30" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D30" s="3"/>
+      <c r="D30" s="3" t="s">
+        <v>260</v>
+      </c>
       <c r="E30" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="F30" s="3"/>
+      <c r="F30" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="G30" s="6">
         <v>0</v>
       </c>
@@ -2978,14 +3321,15 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -2998,8 +3342,8 @@
     <col min="12" max="12" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:12" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>172</v>
       </c>
       <c r="B1" s="9"/>
@@ -3014,7 +3358,7 @@
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
     </row>
-    <row r="3" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>173</v>
       </c>
@@ -3052,14 +3396,16 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="85.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" ht="85.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>182</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="3" t="s">
+        <v>273</v>
+      </c>
       <c r="D4" s="4" t="s">
         <v>184</v>
       </c>
@@ -3069,7 +3415,9 @@
       <c r="F4" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="G4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>288</v>
+      </c>
       <c r="H4" s="3">
         <v>475</v>
       </c>
@@ -3086,14 +3434,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="85.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" ht="85.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>187</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="3" t="s">
+        <v>274</v>
+      </c>
       <c r="D5" s="4" t="s">
         <v>184</v>
       </c>
@@ -3103,7 +3453,9 @@
       <c r="F5" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>287</v>
+      </c>
       <c r="H5" s="3">
         <v>669</v>
       </c>
@@ -3120,14 +3472,16 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" ht="106.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>190</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>275</v>
+      </c>
       <c r="D6" s="4" t="s">
         <v>184</v>
       </c>
@@ -3137,7 +3491,9 @@
       <c r="F6" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="G6" s="3"/>
+      <c r="G6" s="3" t="s">
+        <v>286</v>
+      </c>
       <c r="H6" s="3">
         <v>13107</v>
       </c>
@@ -3154,14 +3510,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>194</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="D7" s="4" t="s">
         <v>184</v>
       </c>
@@ -3171,7 +3529,9 @@
       <c r="F7" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>285</v>
+      </c>
       <c r="H7" s="3">
         <v>47920</v>
       </c>
@@ -3188,14 +3548,16 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="88.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" ht="88.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>197</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="3" t="s">
+        <v>277</v>
+      </c>
       <c r="D8" s="4" t="s">
         <v>184</v>
       </c>
@@ -3205,7 +3567,9 @@
       <c r="F8" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3" t="s">
+        <v>284</v>
+      </c>
       <c r="H8" s="3">
         <v>10.5</v>
       </c>
@@ -3222,14 +3586,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" ht="95.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>201</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="D9" s="4" t="s">
         <v>184</v>
       </c>
@@ -3239,7 +3605,9 @@
       <c r="F9" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="G9" s="3"/>
+      <c r="G9" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H9" s="3">
         <v>5331377</v>
       </c>
@@ -3256,14 +3624,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="99" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" ht="99" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>205</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C10" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>279</v>
+      </c>
       <c r="D10" s="4" t="s">
         <v>207</v>
       </c>
@@ -3273,7 +3643,9 @@
       <c r="F10" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3" t="s">
+        <v>282</v>
+      </c>
       <c r="H10" s="3">
         <v>0</v>
       </c>
@@ -3290,14 +3662,16 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="100.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C11" s="3"/>
+      <c r="C11" s="3" t="s">
+        <v>280</v>
+      </c>
       <c r="D11" s="4" t="s">
         <v>207</v>
       </c>
@@ -3307,7 +3681,9 @@
       <c r="F11" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="G11" s="3"/>
+      <c r="G11" s="3" t="s">
+        <v>281</v>
+      </c>
       <c r="H11" s="3">
         <v>5</v>
       </c>
@@ -3336,7 +3712,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -3344,15 +3720,15 @@
     <col min="4" max="4" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>214</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
     </row>
-    <row r="3" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>173</v>
       </c>
@@ -3366,7 +3742,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>182</v>
       </c>
@@ -3380,7 +3756,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>187</v>
       </c>
@@ -3394,7 +3770,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>190</v>
       </c>
@@ -3408,7 +3784,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>194</v>
       </c>
@@ -3422,7 +3798,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>197</v>
       </c>
@@ -3436,7 +3812,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>201</v>
       </c>
@@ -3450,7 +3826,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>205</v>
       </c>
@@ -3464,7 +3840,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>210</v>
       </c>
@@ -3489,7 +3865,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3500,8 +3876,8 @@
     <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:8" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>226</v>
       </c>
       <c r="B1" s="9"/>
@@ -3512,7 +3888,7 @@
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
     </row>
-    <row r="3" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -3538,8 +3914,8 @@
         <v>217</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>233</v>
       </c>
       <c r="B4" s="9"/>

</xml_diff>